<commit_message>
Refresh 8/08 Meta costs to final values (+3 yen drift)
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-08-09.xlsx
+++ b/data/reports/report-2026-08-09.xlsx
@@ -508,10 +508,10 @@
         <v>281937</v>
       </c>
       <c r="D2" t="n">
-        <v>453941</v>
+        <v>453944</v>
       </c>
       <c r="E2" t="n">
-        <v>214243</v>
+        <v>214240</v>
       </c>
       <c r="F2" t="n">
         <v>22.55</v>
@@ -526,7 +526,7 @@
         <v>32798</v>
       </c>
       <c r="J2" t="n">
-        <v>181445</v>
+        <v>181442</v>
       </c>
     </row>
     <row r="3">
@@ -542,10 +542,10 @@
         <v>749084</v>
       </c>
       <c r="D3" t="n">
-        <v>1291885</v>
+        <v>1291888</v>
       </c>
       <c r="E3" t="n">
-        <v>587714</v>
+        <v>587711</v>
       </c>
       <c r="F3" t="n">
         <v>22.36</v>
@@ -560,7 +560,7 @@
         <v>90742</v>
       </c>
       <c r="J3" t="n">
-        <v>496972</v>
+        <v>496969</v>
       </c>
     </row>
     <row r="4">
@@ -576,10 +576,10 @@
         <v>2027075</v>
       </c>
       <c r="D4" t="n">
-        <v>3383159</v>
+        <v>3383162</v>
       </c>
       <c r="E4" t="n">
-        <v>1583352</v>
+        <v>1583349</v>
       </c>
       <c r="F4" t="n">
         <v>22.64</v>
@@ -594,7 +594,7 @@
         <v>241419</v>
       </c>
       <c r="J4" t="n">
-        <v>1341933</v>
+        <v>1341930</v>
       </c>
     </row>
     <row r="5">
@@ -610,10 +610,10 @@
         <v>11255315</v>
       </c>
       <c r="D5" t="n">
-        <v>15351146</v>
+        <v>15351149</v>
       </c>
       <c r="E5" t="n">
-        <v>11134540</v>
+        <v>11134537</v>
       </c>
       <c r="F5" t="n">
         <v>29.5</v>
@@ -628,7 +628,7 @@
         <v>1302819</v>
       </c>
       <c r="J5" t="n">
-        <v>9831721</v>
+        <v>9831718</v>
       </c>
     </row>
   </sheetData>
@@ -758,10 +758,10 @@
         <v>263250</v>
       </c>
       <c r="D2" t="n">
-        <v>556695</v>
+        <v>556696</v>
       </c>
       <c r="E2" t="n">
-        <v>557732</v>
+        <v>557731</v>
       </c>
       <c r="F2" t="n">
         <v>2.47</v>
@@ -776,16 +776,16 @@
         <v>186264</v>
       </c>
       <c r="J2" t="n">
-        <v>61895</v>
+        <v>61894</v>
       </c>
       <c r="K2" t="n">
         <v>33.2</v>
       </c>
       <c r="L2" t="n">
-        <v>261082</v>
+        <v>261081</v>
       </c>
       <c r="M2" t="n">
-        <v>1920945</v>
+        <v>1920944</v>
       </c>
       <c r="N2" t="n">
         <v>350</v>
@@ -1117,7 +1117,7 @@
         <v>100</v>
       </c>
       <c r="O8" t="n">
-        <v>23000</v>
+        <v>26000</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -1138,10 +1138,10 @@
         <v>103411</v>
       </c>
       <c r="D9" t="n">
-        <v>210410</v>
+        <v>210411</v>
       </c>
       <c r="E9" t="n">
-        <v>70386</v>
+        <v>70385</v>
       </c>
       <c r="F9" t="n">
         <v>1.83</v>
@@ -1156,16 +1156,16 @@
         <v>33864</v>
       </c>
       <c r="J9" t="n">
-        <v>-3144</v>
+        <v>-3145</v>
       </c>
       <c r="K9" t="n">
         <v>-9.300000000000001</v>
       </c>
       <c r="L9" t="n">
-        <v>20465</v>
+        <v>20464</v>
       </c>
       <c r="M9" t="n">
-        <v>749523</v>
+        <v>749522</v>
       </c>
       <c r="N9" t="n">
         <v>79</v>
@@ -1300,10 +1300,10 @@
         <v>65868</v>
       </c>
       <c r="D12" t="n">
-        <v>118085</v>
+        <v>118086</v>
       </c>
       <c r="E12" t="n">
-        <v>12191</v>
+        <v>12190</v>
       </c>
       <c r="F12" t="n">
         <v>1.66</v>
@@ -1318,16 +1318,16 @@
         <v>11960</v>
       </c>
       <c r="J12" t="n">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="K12" t="n">
         <v>4.9</v>
       </c>
       <c r="L12" t="n">
-        <v>-2801</v>
+        <v>-2802</v>
       </c>
       <c r="M12" t="n">
-        <v>559305</v>
+        <v>559304</v>
       </c>
       <c r="N12" t="n">
         <v>33</v>
@@ -1551,7 +1551,7 @@
         <v>26</v>
       </c>
       <c r="O16" t="n">
-        <v>12500</v>
+        <v>15000</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
@@ -2881,16 +2881,16 @@
         <v>950121</v>
       </c>
       <c r="D17" t="n">
-        <v>453941</v>
+        <v>453944</v>
       </c>
       <c r="E17" t="n">
-        <v>214398</v>
+        <v>214395</v>
       </c>
       <c r="F17" t="n">
         <v>22.57</v>
       </c>
       <c r="G17" t="n">
-        <v>196073</v>
+        <v>196072</v>
       </c>
     </row>
   </sheetData>

</xml_diff>